<commit_message>
feat(sg): add initial list of services
</commit_message>
<xml_diff>
--- a/django/kt_sg/import/Services_SG.xlsx
+++ b/django/kt_sg/import/Services_SG.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
   <si>
     <t xml:space="preserve">Typ</t>
   </si>
@@ -279,6 +279,12 @@
   </si>
   <si>
     <t xml:space="preserve">Waldkirch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koordinationsstelle Bau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coordination</t>
   </si>
   <si>
     <t xml:space="preserve">Statistik Schweiz - BFS</t>
@@ -333,7 +339,7 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="12"/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -394,16 +400,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -598,11 +608,21 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K76"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="5.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="4.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="10.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="7.69"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16375" min="12" style="1" width="8.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16376" style="1" width="11.53"/>
   </cols>
   <sheetData>
@@ -642,11 +662,13 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0"/>
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J2" s="0" t="n">
+      <c r="J2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K2" s="1" t="n">
@@ -654,11 +676,13 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0"/>
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="0" t="n">
+      <c r="J3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K3" s="1" t="n">
@@ -666,11 +690,13 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0"/>
+      <c r="A4" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="0" t="n">
+      <c r="J4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K4" s="1" t="n">
@@ -678,11 +704,13 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0"/>
+      <c r="A5" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="0" t="n">
+      <c r="J5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K5" s="1" t="n">
@@ -690,11 +718,13 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0"/>
+      <c r="A6" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="0" t="n">
+      <c r="J6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K6" s="1" t="n">
@@ -702,11 +732,13 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0"/>
+      <c r="A7" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="0" t="n">
+      <c r="J7" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K7" s="1" t="n">
@@ -714,11 +746,13 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0"/>
+      <c r="A8" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="0" t="n">
+      <c r="J8" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K8" s="1" t="n">
@@ -726,11 +760,13 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0"/>
+      <c r="A9" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="0" t="n">
+      <c r="J9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K9" s="1" t="n">
@@ -738,11 +774,13 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0"/>
+      <c r="A10" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="0" t="n">
+      <c r="J10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K10" s="1" t="n">
@@ -750,11 +788,13 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0"/>
+      <c r="A11" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J11" s="0" t="n">
+      <c r="J11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K11" s="1" t="n">
@@ -762,11 +802,13 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0"/>
+      <c r="A12" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J12" s="0" t="n">
+      <c r="J12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K12" s="1" t="n">
@@ -774,11 +816,13 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0"/>
+      <c r="A13" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B13" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J13" s="0" t="n">
+      <c r="J13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K13" s="1" t="n">
@@ -786,11 +830,13 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0"/>
+      <c r="A14" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B14" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J14" s="0" t="n">
+      <c r="J14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K14" s="1" t="n">
@@ -798,11 +844,13 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0"/>
+      <c r="A15" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B15" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J15" s="0" t="n">
+      <c r="J15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K15" s="1" t="n">
@@ -810,11 +858,13 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0"/>
+      <c r="A16" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B16" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="J16" s="0" t="n">
+      <c r="J16" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K16" s="1" t="n">
@@ -822,11 +872,13 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0"/>
+      <c r="A17" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J17" s="0" t="n">
+      <c r="J17" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K17" s="1" t="n">
@@ -834,11 +886,13 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0"/>
+      <c r="A18" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J18" s="0" t="n">
+      <c r="J18" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K18" s="1" t="n">
@@ -846,11 +900,13 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0"/>
+      <c r="A19" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B19" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J19" s="0" t="n">
+      <c r="J19" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K19" s="1" t="n">
@@ -858,11 +914,13 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0"/>
+      <c r="A20" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B20" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="J20" s="0" t="n">
+      <c r="J20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K20" s="1" t="n">
@@ -870,11 +928,13 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0"/>
+      <c r="A21" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B21" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="J21" s="0" t="n">
+      <c r="J21" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K21" s="1" t="n">
@@ -882,11 +942,13 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0"/>
+      <c r="A22" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B22" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J22" s="0" t="n">
+      <c r="J22" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K22" s="1" t="n">
@@ -894,11 +956,13 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0"/>
+      <c r="A23" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="J23" s="0" t="n">
+      <c r="J23" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K23" s="1" t="n">
@@ -906,11 +970,13 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0"/>
+      <c r="A24" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B24" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="J24" s="0" t="n">
+      <c r="J24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K24" s="1" t="n">
@@ -918,11 +984,13 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0"/>
+      <c r="A25" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B25" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="J25" s="0" t="n">
+      <c r="J25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K25" s="1" t="n">
@@ -930,11 +998,13 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0"/>
+      <c r="A26" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B26" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J26" s="0" t="n">
+      <c r="J26" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K26" s="1" t="n">
@@ -942,11 +1012,13 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0"/>
+      <c r="A27" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B27" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J27" s="0" t="n">
+      <c r="J27" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K27" s="1" t="n">
@@ -954,11 +1026,13 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0"/>
+      <c r="A28" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B28" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="J28" s="0" t="n">
+      <c r="J28" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K28" s="1" t="n">
@@ -966,11 +1040,13 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0"/>
+      <c r="A29" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B29" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J29" s="0" t="n">
+      <c r="J29" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K29" s="1" t="n">
@@ -978,11 +1054,13 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0"/>
+      <c r="A30" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B30" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="J30" s="0" t="n">
+      <c r="J30" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K30" s="1" t="n">
@@ -990,11 +1068,13 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0"/>
+      <c r="A31" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B31" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="J31" s="0" t="n">
+      <c r="J31" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K31" s="1" t="n">
@@ -1002,11 +1082,13 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0"/>
+      <c r="A32" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B32" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J32" s="0" t="n">
+      <c r="J32" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K32" s="1" t="n">
@@ -1014,11 +1096,13 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0"/>
+      <c r="A33" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B33" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J33" s="0" t="n">
+      <c r="J33" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K33" s="1" t="n">
@@ -1026,11 +1110,13 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0"/>
+      <c r="A34" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B34" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J34" s="0" t="n">
+      <c r="J34" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K34" s="1" t="n">
@@ -1038,11 +1124,13 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0"/>
+      <c r="A35" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B35" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J35" s="0" t="n">
+      <c r="J35" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K35" s="1" t="n">
@@ -1050,11 +1138,13 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0"/>
+      <c r="A36" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B36" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J36" s="0" t="n">
+      <c r="J36" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K36" s="1" t="n">
@@ -1062,11 +1152,13 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0"/>
+      <c r="A37" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B37" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J37" s="0" t="n">
+      <c r="J37" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K37" s="1" t="n">
@@ -1074,11 +1166,13 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0"/>
+      <c r="A38" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B38" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="J38" s="0" t="n">
+      <c r="J38" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K38" s="1" t="n">
@@ -1086,11 +1180,13 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0"/>
+      <c r="A39" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B39" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J39" s="0" t="n">
+      <c r="J39" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K39" s="1" t="n">
@@ -1098,11 +1194,13 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0"/>
+      <c r="A40" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B40" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="J40" s="0" t="n">
+      <c r="J40" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K40" s="1" t="n">
@@ -1110,11 +1208,13 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0"/>
+      <c r="A41" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B41" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="J41" s="0" t="n">
+      <c r="J41" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K41" s="1" t="n">
@@ -1122,11 +1222,13 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0"/>
+      <c r="A42" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B42" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="J42" s="0" t="n">
+      <c r="J42" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K42" s="1" t="n">
@@ -1134,11 +1236,13 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0"/>
+      <c r="A43" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B43" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="J43" s="0" t="n">
+      <c r="J43" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K43" s="1" t="n">
@@ -1146,11 +1250,13 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0"/>
+      <c r="A44" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B44" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="J44" s="0" t="n">
+      <c r="J44" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K44" s="1" t="n">
@@ -1158,11 +1264,13 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0"/>
+      <c r="A45" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B45" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="J45" s="0" t="n">
+      <c r="J45" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K45" s="1" t="n">
@@ -1170,11 +1278,13 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0"/>
+      <c r="A46" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B46" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="J46" s="0" t="n">
+      <c r="J46" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K46" s="1" t="n">
@@ -1182,11 +1292,13 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0"/>
+      <c r="A47" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B47" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J47" s="0" t="n">
+      <c r="J47" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K47" s="1" t="n">
@@ -1194,11 +1306,13 @@
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0"/>
+      <c r="A48" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B48" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="J48" s="0" t="n">
+      <c r="J48" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K48" s="1" t="n">
@@ -1206,11 +1320,13 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0"/>
+      <c r="A49" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B49" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="J49" s="0" t="n">
+      <c r="J49" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K49" s="1" t="n">
@@ -1218,11 +1334,13 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0"/>
+      <c r="A50" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B50" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="J50" s="0" t="n">
+      <c r="J50" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K50" s="1" t="n">
@@ -1230,11 +1348,13 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0"/>
+      <c r="A51" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B51" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="J51" s="0" t="n">
+      <c r="J51" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K51" s="1" t="n">
@@ -1242,11 +1362,13 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0"/>
+      <c r="A52" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B52" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="J52" s="0" t="n">
+      <c r="J52" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K52" s="1" t="n">
@@ -1254,11 +1376,13 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="0"/>
+      <c r="A53" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B53" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="J53" s="0" t="n">
+      <c r="J53" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K53" s="1" t="n">
@@ -1266,11 +1390,13 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="0"/>
+      <c r="A54" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B54" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="J54" s="0" t="n">
+      <c r="J54" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K54" s="1" t="n">
@@ -1278,11 +1404,13 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="0"/>
+      <c r="A55" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B55" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="J55" s="0" t="n">
+      <c r="J55" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K55" s="1" t="n">
@@ -1290,11 +1418,13 @@
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="0"/>
+      <c r="A56" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B56" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="J56" s="0" t="n">
+      <c r="J56" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K56" s="1" t="n">
@@ -1302,11 +1432,13 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="0"/>
+      <c r="A57" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B57" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="J57" s="0" t="n">
+      <c r="J57" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K57" s="1" t="n">
@@ -1314,11 +1446,13 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0"/>
+      <c r="A58" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B58" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J58" s="0" t="n">
+      <c r="J58" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K58" s="1" t="n">
@@ -1326,11 +1460,13 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="0"/>
+      <c r="A59" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B59" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="J59" s="0" t="n">
+      <c r="J59" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K59" s="1" t="n">
@@ -1338,11 +1474,13 @@
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="0"/>
+      <c r="A60" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B60" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="J60" s="0" t="n">
+      <c r="J60" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K60" s="1" t="n">
@@ -1350,11 +1488,13 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0"/>
+      <c r="A61" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B61" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="J61" s="0" t="n">
+      <c r="J61" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K61" s="1" t="n">
@@ -1362,11 +1502,13 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0"/>
+      <c r="A62" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B62" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="J62" s="0" t="n">
+      <c r="J62" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K62" s="1" t="n">
@@ -1374,11 +1516,13 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0"/>
+      <c r="A63" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B63" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="J63" s="0" t="n">
+      <c r="J63" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K63" s="1" t="n">
@@ -1386,11 +1530,13 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0"/>
+      <c r="A64" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B64" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="J64" s="0" t="n">
+      <c r="J64" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K64" s="1" t="n">
@@ -1398,11 +1544,13 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0"/>
+      <c r="A65" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B65" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="J65" s="0" t="n">
+      <c r="J65" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K65" s="1" t="n">
@@ -1410,11 +1558,13 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0"/>
+      <c r="A66" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B66" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="J66" s="0" t="n">
+      <c r="J66" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K66" s="1" t="n">
@@ -1422,11 +1572,13 @@
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="0"/>
+      <c r="A67" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B67" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="J67" s="0" t="n">
+      <c r="J67" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K67" s="1" t="n">
@@ -1434,11 +1586,13 @@
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0"/>
+      <c r="A68" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B68" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="J68" s="0" t="n">
+      <c r="J68" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K68" s="1" t="n">
@@ -1446,11 +1600,13 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0"/>
+      <c r="A69" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B69" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="J69" s="0" t="n">
+      <c r="J69" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K69" s="1" t="n">
@@ -1458,11 +1614,13 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="0"/>
+      <c r="A70" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B70" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="J70" s="0" t="n">
+      <c r="J70" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K70" s="1" t="n">
@@ -1470,11 +1628,13 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="0"/>
+      <c r="A71" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B71" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="J71" s="0" t="n">
+      <c r="J71" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K71" s="1" t="n">
@@ -1482,11 +1642,13 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0"/>
+      <c r="A72" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B72" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="J72" s="0" t="n">
+      <c r="J72" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K72" s="1" t="n">
@@ -1494,11 +1656,13 @@
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0"/>
+      <c r="A73" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B73" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="J73" s="0" t="n">
+      <c r="J73" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K73" s="1" t="n">
@@ -1506,11 +1670,13 @@
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="0"/>
+      <c r="A74" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B74" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="J74" s="0" t="n">
+      <c r="J74" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K74" s="1" t="n">
@@ -1518,11 +1684,13 @@
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="0"/>
+      <c r="A75" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B75" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J75" s="0" t="n">
+      <c r="J75" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K75" s="1" t="n">
@@ -1530,15 +1698,31 @@
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="0"/>
+      <c r="A76" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="B76" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="J76" s="0" t="n">
+      <c r="J76" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K76" s="1" t="n">
         <v>3444</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J77" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1560,42 +1744,42 @@
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="91.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="91.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
-        <v>86</v>
+      <c r="A1" s="4" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>87</v>
+      <c r="A2" s="4" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>88</v>
+      <c r="A3" s="3" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>89</v>
+      <c r="A4" s="3" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>90</v>
+      <c r="A6" s="4" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>91</v>
+      <c r="A8" s="3" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>92</v>
+      <c r="A9" s="5" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(sg): integrate and configure distribution module
Related to https://jira.sg.ch/browse/EBAU-168
</commit_message>
<xml_diff>
--- a/django/kt_sg/import/Services_SG.xlsx
+++ b/django/kt_sg/import/Services_SG.xlsx
@@ -9,7 +9,6 @@
   </bookViews>
   <sheets>
     <sheet name="Daten" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Metadaten" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="161">
   <si>
     <t xml:space="preserve">Typ</t>
   </si>
@@ -56,6 +55,9 @@
     <t xml:space="preserve">BFS Nr</t>
   </si>
   <si>
+    <t xml:space="preserve">Meta</t>
+  </si>
+  <si>
     <t xml:space="preserve">Häggenschwil</t>
   </si>
   <si>
@@ -290,6 +292,9 @@
     <t xml:space="preserve">AFU-BS-AR Abfall und Rohstoffe</t>
   </si>
   <si>
+    <t xml:space="preserve">{"distribution-group": "bud"}</t>
+  </si>
+  <si>
     <t xml:space="preserve">AFU-BS-BA Boden und Altlasten</t>
   </si>
   <si>
@@ -389,12 +394,18 @@
     <t xml:space="preserve">AfKU-AR Archäologie</t>
   </si>
   <si>
+    <t xml:space="preserve">{"distribution-group": "di"}</t>
+  </si>
+  <si>
     <t xml:space="preserve">AfKU-KDP Denkmalpflege</t>
   </si>
   <si>
     <t xml:space="preserve">AVSV-Lab Kantonales Labor</t>
   </si>
   <si>
+    <t xml:space="preserve">{"distribution-group": "gd"}</t>
+  </si>
+  <si>
     <t xml:space="preserve">AVSV-LMI Lebensmittelinspektorat</t>
   </si>
   <si>
@@ -407,6 +418,9 @@
     <t xml:space="preserve">AfMZ-BVS Infrastruktur Zivilschutz</t>
   </si>
   <si>
+    <t xml:space="preserve">{"distribution-group": "sjd"}</t>
+  </si>
+  <si>
     <t xml:space="preserve">GVSG-BS Brandschutz</t>
   </si>
   <si>
@@ -489,27 +503,6 @@
   </si>
   <si>
     <t xml:space="preserve">AB Appenzeller Bahnen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Statistik Schweiz - BFS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Historisiertes Gemeindeverzeichnis der Schweiz - Abfragetool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Datengrundlage 12.09.1848 - 01.01.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">© 2026 Bundesamt für Statistik BFS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gemeindestand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Erstellungsdatum: 11.02.2026 09:23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gemeindestand am 01.01.2026, basierend auf offiziellem Gemeindestand vom 01.01.2026. (2’110 Einträge)</t>
   </si>
 </sst>
 </file>
@@ -519,7 +512,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -546,13 +539,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -604,7 +590,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -619,14 +605,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -812,7 +790,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K1048576"/>
+  <dimension ref="A1:L1048576"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.77"/>
@@ -826,7 +804,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="10.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="7.69"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16375" min="12" style="1" width="8.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="23.37"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16375" min="13" style="1" width="8.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16376" style="1" width="11.53"/>
   </cols>
   <sheetData>
@@ -864,13 +843,16 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J2" s="1" t="n">
         <v>0</v>
@@ -884,7 +866,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J3" s="1" t="n">
         <v>0</v>
@@ -898,7 +880,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J4" s="1" t="n">
         <v>0</v>
@@ -912,7 +894,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J5" s="1" t="n">
         <v>0</v>
@@ -926,7 +908,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J6" s="1" t="n">
         <v>0</v>
@@ -940,7 +922,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J7" s="1" t="n">
         <v>0</v>
@@ -954,7 +936,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J8" s="1" t="n">
         <v>0</v>
@@ -968,7 +950,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J9" s="1" t="n">
         <v>0</v>
@@ -982,7 +964,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J10" s="1" t="n">
         <v>0</v>
@@ -996,7 +978,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J11" s="1" t="n">
         <v>0</v>
@@ -1010,7 +992,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J12" s="1" t="n">
         <v>0</v>
@@ -1024,7 +1006,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J13" s="1" t="n">
         <v>0</v>
@@ -1038,7 +1020,7 @@
         <v>1</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J14" s="1" t="n">
         <v>0</v>
@@ -1052,7 +1034,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J15" s="1" t="n">
         <v>0</v>
@@ -1066,7 +1048,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J16" s="1" t="n">
         <v>0</v>
@@ -1080,7 +1062,7 @@
         <v>1</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J17" s="1" t="n">
         <v>0</v>
@@ -1094,7 +1076,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J18" s="1" t="n">
         <v>0</v>
@@ -1108,7 +1090,7 @@
         <v>1</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J19" s="1" t="n">
         <v>0</v>
@@ -1122,7 +1104,7 @@
         <v>1</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J20" s="1" t="n">
         <v>0</v>
@@ -1136,7 +1118,7 @@
         <v>1</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J21" s="1" t="n">
         <v>0</v>
@@ -1150,7 +1132,7 @@
         <v>1</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="J22" s="1" t="n">
         <v>0</v>
@@ -1164,7 +1146,7 @@
         <v>1</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J23" s="1" t="n">
         <v>0</v>
@@ -1178,7 +1160,7 @@
         <v>1</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J24" s="1" t="n">
         <v>0</v>
@@ -1192,7 +1174,7 @@
         <v>1</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J25" s="1" t="n">
         <v>0</v>
@@ -1206,7 +1188,7 @@
         <v>1</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J26" s="1" t="n">
         <v>0</v>
@@ -1220,7 +1202,7 @@
         <v>1</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J27" s="1" t="n">
         <v>0</v>
@@ -1234,7 +1216,7 @@
         <v>1</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J28" s="1" t="n">
         <v>0</v>
@@ -1248,7 +1230,7 @@
         <v>1</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J29" s="1" t="n">
         <v>0</v>
@@ -1262,7 +1244,7 @@
         <v>1</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J30" s="1" t="n">
         <v>0</v>
@@ -1276,7 +1258,7 @@
         <v>1</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J31" s="1" t="n">
         <v>0</v>
@@ -1290,7 +1272,7 @@
         <v>1</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J32" s="1" t="n">
         <v>0</v>
@@ -1304,7 +1286,7 @@
         <v>1</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J33" s="1" t="n">
         <v>0</v>
@@ -1318,7 +1300,7 @@
         <v>1</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J34" s="1" t="n">
         <v>0</v>
@@ -1332,7 +1314,7 @@
         <v>1</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J35" s="1" t="n">
         <v>0</v>
@@ -1346,7 +1328,7 @@
         <v>1</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J36" s="1" t="n">
         <v>0</v>
@@ -1360,7 +1342,7 @@
         <v>1</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J37" s="1" t="n">
         <v>0</v>
@@ -1374,7 +1356,7 @@
         <v>1</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J38" s="1" t="n">
         <v>0</v>
@@ -1388,7 +1370,7 @@
         <v>1</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J39" s="1" t="n">
         <v>0</v>
@@ -1402,7 +1384,7 @@
         <v>1</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J40" s="1" t="n">
         <v>0</v>
@@ -1416,7 +1398,7 @@
         <v>1</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J41" s="1" t="n">
         <v>0</v>
@@ -1430,7 +1412,7 @@
         <v>1</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J42" s="1" t="n">
         <v>0</v>
@@ -1444,7 +1426,7 @@
         <v>1</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J43" s="1" t="n">
         <v>0</v>
@@ -1458,7 +1440,7 @@
         <v>1</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J44" s="1" t="n">
         <v>0</v>
@@ -1472,7 +1454,7 @@
         <v>1</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J45" s="1" t="n">
         <v>0</v>
@@ -1486,7 +1468,7 @@
         <v>1</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J46" s="1" t="n">
         <v>0</v>
@@ -1500,7 +1482,7 @@
         <v>1</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J47" s="1" t="n">
         <v>0</v>
@@ -1514,7 +1496,7 @@
         <v>1</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J48" s="1" t="n">
         <v>0</v>
@@ -1528,7 +1510,7 @@
         <v>1</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J49" s="1" t="n">
         <v>0</v>
@@ -1542,7 +1524,7 @@
         <v>1</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J50" s="1" t="n">
         <v>0</v>
@@ -1556,7 +1538,7 @@
         <v>1</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J51" s="1" t="n">
         <v>0</v>
@@ -1570,7 +1552,7 @@
         <v>1</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J52" s="1" t="n">
         <v>0</v>
@@ -1584,7 +1566,7 @@
         <v>1</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J53" s="1" t="n">
         <v>0</v>
@@ -1598,7 +1580,7 @@
         <v>1</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J54" s="1" t="n">
         <v>0</v>
@@ -1612,7 +1594,7 @@
         <v>1</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J55" s="1" t="n">
         <v>0</v>
@@ -1626,7 +1608,7 @@
         <v>1</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J56" s="1" t="n">
         <v>0</v>
@@ -1640,7 +1622,7 @@
         <v>1</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J57" s="1" t="n">
         <v>0</v>
@@ -1654,7 +1636,7 @@
         <v>1</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J58" s="1" t="n">
         <v>0</v>
@@ -1668,7 +1650,7 @@
         <v>1</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J59" s="1" t="n">
         <v>0</v>
@@ -1682,7 +1664,7 @@
         <v>1</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J60" s="1" t="n">
         <v>0</v>
@@ -1696,7 +1678,7 @@
         <v>1</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J61" s="1" t="n">
         <v>0</v>
@@ -1710,7 +1692,7 @@
         <v>1</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J62" s="1" t="n">
         <v>0</v>
@@ -1724,7 +1706,7 @@
         <v>1</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J63" s="1" t="n">
         <v>0</v>
@@ -1738,7 +1720,7 @@
         <v>1</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J64" s="1" t="n">
         <v>0</v>
@@ -1752,7 +1734,7 @@
         <v>1</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J65" s="1" t="n">
         <v>0</v>
@@ -1766,7 +1748,7 @@
         <v>1</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J66" s="1" t="n">
         <v>0</v>
@@ -1780,7 +1762,7 @@
         <v>1</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J67" s="1" t="n">
         <v>0</v>
@@ -1794,7 +1776,7 @@
         <v>1</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J68" s="1" t="n">
         <v>0</v>
@@ -1808,7 +1790,7 @@
         <v>1</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J69" s="1" t="n">
         <v>0</v>
@@ -1822,7 +1804,7 @@
         <v>1</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J70" s="1" t="n">
         <v>0</v>
@@ -1836,7 +1818,7 @@
         <v>1</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J71" s="1" t="n">
         <v>0</v>
@@ -1850,7 +1832,7 @@
         <v>1</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J72" s="1" t="n">
         <v>0</v>
@@ -1864,7 +1846,7 @@
         <v>1</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J73" s="1" t="n">
         <v>0</v>
@@ -1878,7 +1860,7 @@
         <v>1</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J74" s="1" t="n">
         <v>0</v>
@@ -1892,7 +1874,7 @@
         <v>1</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J75" s="1" t="n">
         <v>0</v>
@@ -1906,7 +1888,7 @@
         <v>1</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J76" s="1" t="n">
         <v>0</v>
@@ -1920,10 +1902,10 @@
         <v>2</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J77" s="1" t="n">
         <v>0</v>
@@ -1934,10 +1916,13 @@
         <v>3</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J78" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L78" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1945,10 +1930,13 @@
         <v>3</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J79" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L79" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1956,10 +1944,13 @@
         <v>3</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="J80" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L80" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1967,10 +1958,13 @@
         <v>3</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J81" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L81" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1978,10 +1972,13 @@
         <v>3</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="J82" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L82" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1989,10 +1986,13 @@
         <v>3</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="J83" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L83" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2000,10 +2000,13 @@
         <v>3</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J84" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L84" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2011,10 +2014,13 @@
         <v>3</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J85" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L85" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2022,10 +2028,13 @@
         <v>3</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="J86" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L86" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2033,10 +2042,13 @@
         <v>3</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J87" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L87" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2044,10 +2056,13 @@
         <v>3</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J88" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L88" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2055,10 +2070,13 @@
         <v>3</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="J89" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L89" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2066,10 +2084,13 @@
         <v>3</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="J90" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L90" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2077,10 +2098,13 @@
         <v>3</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J91" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L91" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2088,10 +2112,13 @@
         <v>3</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J92" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L92" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2099,10 +2126,13 @@
         <v>3</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J93" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L93" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2110,10 +2140,13 @@
         <v>3</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J94" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L94" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2121,10 +2154,13 @@
         <v>3</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J95" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L95" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2132,10 +2168,13 @@
         <v>3</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="J96" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L96" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2143,10 +2182,13 @@
         <v>3</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J97" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L97" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2154,10 +2196,13 @@
         <v>3</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="J98" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L98" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2165,10 +2210,13 @@
         <v>3</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J99" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L99" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2176,10 +2224,13 @@
         <v>3</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J100" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L100" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2187,10 +2238,13 @@
         <v>3</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="J101" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L101" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2198,10 +2252,13 @@
         <v>3</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="J102" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L102" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2209,10 +2266,13 @@
         <v>3</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="J103" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L103" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2220,10 +2280,13 @@
         <v>3</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="J104" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L104" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2231,10 +2294,13 @@
         <v>3</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J105" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L105" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2242,10 +2308,13 @@
         <v>3</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="J106" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L106" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2253,10 +2322,13 @@
         <v>3</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="J107" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L107" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2264,10 +2336,13 @@
         <v>3</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="J108" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L108" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2275,10 +2350,13 @@
         <v>3</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J109" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L109" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2286,10 +2364,13 @@
         <v>3</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="J110" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L110" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2297,10 +2378,13 @@
         <v>3</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="J111" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L111" s="1" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2308,10 +2392,13 @@
         <v>3</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="J112" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L112" s="1" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2319,10 +2406,13 @@
         <v>3</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="J113" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L113" s="1" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2330,10 +2420,13 @@
         <v>3</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="J114" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L114" s="1" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2341,10 +2434,13 @@
         <v>3</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="J115" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L115" s="1" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2352,10 +2448,13 @@
         <v>3</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J116" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L116" s="1" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2363,10 +2462,13 @@
         <v>3</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="J117" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L117" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2374,10 +2476,13 @@
         <v>3</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="J118" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L118" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2385,10 +2490,13 @@
         <v>3</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="J119" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L119" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2396,10 +2504,13 @@
         <v>3</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="J120" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L120" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2407,10 +2518,13 @@
         <v>3</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="J121" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L121" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2418,10 +2532,13 @@
         <v>3</v>
       </c>
       <c r="B122" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="J122" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L122" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="J122" s="1" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2429,10 +2546,13 @@
         <v>3</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="J123" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L123" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2440,10 +2560,13 @@
         <v>3</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="J124" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L124" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2451,10 +2574,13 @@
         <v>3</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="J125" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L125" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2462,10 +2588,13 @@
         <v>3</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="J126" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L126" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2473,10 +2602,13 @@
         <v>3</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="J127" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L127" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2484,10 +2616,13 @@
         <v>3</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="J128" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L128" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2495,10 +2630,13 @@
         <v>3</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="J129" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L129" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2506,10 +2644,13 @@
         <v>3</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="J130" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="L130" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2517,7 +2658,7 @@
         <v>4</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="J131" s="1" t="n">
         <v>0</v>
@@ -2528,7 +2669,7 @@
         <v>4</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="J132" s="1" t="n">
         <v>0</v>
@@ -2539,7 +2680,7 @@
         <v>5</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J133" s="1" t="n">
         <v>0</v>
@@ -2550,7 +2691,7 @@
         <v>5</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="J134" s="1" t="n">
         <v>0</v>
@@ -2561,7 +2702,7 @@
         <v>5</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="J135" s="1" t="n">
         <v>0</v>
@@ -2572,7 +2713,7 @@
         <v>5</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="J136" s="1" t="n">
         <v>0</v>
@@ -2583,7 +2724,7 @@
         <v>5</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="J137" s="1" t="n">
         <v>0</v>
@@ -2594,7 +2735,7 @@
         <v>5</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J138" s="1" t="n">
         <v>0</v>
@@ -2605,7 +2746,7 @@
         <v>5</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="J139" s="1" t="n">
         <v>0</v>
@@ -2616,7 +2757,7 @@
         <v>5</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="J140" s="1" t="n">
         <v>0</v>
@@ -2627,7 +2768,7 @@
         <v>5</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="J141" s="1" t="n">
         <v>0</v>
@@ -2638,7 +2779,7 @@
         <v>5</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="J142" s="1" t="n">
         <v>0</v>
@@ -2649,7 +2790,7 @@
         <v>5</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="J143" s="1" t="n">
         <v>0</v>
@@ -2660,7 +2801,7 @@
         <v>5</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="J144" s="1" t="n">
         <v>0</v>
@@ -2671,7 +2812,7 @@
         <v>5</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="J145" s="1" t="n">
         <v>0</v>
@@ -2708,61 +2849,4 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="91.43"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>162</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
chore(sg): add new services from excel list
</commit_message>
<xml_diff>
--- a/django/kt_sg/import/Services_SG.xlsx
+++ b/django/kt_sg/import/Services_SG.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
   <si>
     <t xml:space="preserve">Typ</t>
   </si>
@@ -281,10 +281,214 @@
     <t xml:space="preserve">Waldkirch</t>
   </si>
   <si>
-    <t xml:space="preserve">Koordinationsstelle Bau</t>
+    <t xml:space="preserve">KSB Koordinationsstelle Bau</t>
   </si>
   <si>
     <t xml:space="preserve">coordination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFU-BS-AR Abfall und Rohstoffe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFU-BS-BA Boden und Altlasten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFU-BS-LW Landwirtschaftlicher Umweltschutz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFU-IG-B1 Betriebe 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFU-IG-B2 Betriebe 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFU-IG-LU Luftqualität</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFU-RU-RD Rechtsdienst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFU-RU-UVP UVP und Planbeurteilung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFU-RU-NIS NIS Fachstelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AREG-BAB Bauen ausserhalb Bauzonen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AREG-KP Kantonale Planung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AREG-OP Ortsplanung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AREG-VM Vermessung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AREG-GI-GSM Geoservice-Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AREG-ZD Zentrale Dienste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBA-MUP-SP Spezialprojekte mit Fachstelle Immissionen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBA-MUP-VP Verkehrsplanung mit Fachstelle Fuss- und Veloverkehr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBA-SUK-KB Kunstbauten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBA-SUK-SN Strassenbau Neuhaus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBA-SUK-SB Strassenbau St. Gallen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBA-SI-EB Erhaltungsplanung+Bewilligungen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBA-KI Kantonsingenieur-Büro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBA-GG Grundstückgeschäfte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWE-EK Energie und Klima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWE-GG-AW Abwasser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWE-GG-GW Grundwasser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWE-GG-WK Wasserkraft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWE-RH Rhein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWE-WN-GG Gemeindegewässer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWE-WN-KG Kantonsgewässer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWE-WN-NG Naturgefahren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GS-RA-T1 Team 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GS-RA-T2 Team 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AfKU-AR Archäologie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AfKU-KDP Denkmalpflege</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVSV-Lab Kantonales Labor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVSV-LMI Lebensmittelinspektorat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVSV-VET Veterinärdienst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GS-KtsAPO Kantonsapotheke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AfMZ-BVS Infrastruktur Zivilschutz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GVSG-BS Brandschutz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GVSG-PN Prävention Naturgefahren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAPO-VEPO-VT Verkehrstechnik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAPO-SIPO-SIWAS Sicherheitsfirmen, Waffen,  Sprengstoffe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">StVA-SCH Schiffahrt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANJF-F Fischerei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANJF-J Jagd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANJF-NL Natur- und Landschaftschutz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWA-Insp Arbeitsinspektorat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWA-Stao Standortförderung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KFA-WP Waldrecht und Planung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AöV Amt für öffentlichen Verkehr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LwA-SV/BR Strukturverbesserung / Bodenrecht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUVA Schweizerische Unfallversicherungsanstalt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">agriss Stiftung AgriSicherheit Schweiz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASTRA Bundesamt für Strassen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESTI Eidgenössisches Starkstrominspektorat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BAFU Bundesamt für Umwelt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SBB Schweizerische Bundesbahnen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BAZL Bundesamt für Zivilluftfahrt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BAV Bundesamt für Verkehr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BFE Bundesamt für Energie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EJPD Eidgenössischens Justiz und Polizei Departement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VBS Eidgenösssiches Departement für Verteidigung, Bevölkerungsschutz und Sport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESO-18 Kreis 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESO-19 Kreis 19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOB Schweizerische Südostbahn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AB Appenzeller Bahnen</t>
   </si>
   <si>
     <t xml:space="preserve">Statistik Schweiz - BFS</t>
@@ -413,16 +617,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -608,14 +812,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:K1048576"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="51.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="5.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="5.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="4.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.97"/>
@@ -1725,6 +1929,776 @@
         <v>0</v>
       </c>
     </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="J78" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="J79" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="J80" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="J81" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="J82" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="J83" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="J84" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="J85" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J86" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="J87" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="J88" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="J89" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="J90" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="J91" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="J92" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J93" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="J94" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J95" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="J96" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="J97" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="J98" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="J99" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="J100" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="J101" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="J102" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="J103" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J104" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="J105" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="J106" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="J107" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="J108" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="J109" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="J110" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="J111" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="J112" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J113" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="J114" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="J115" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="J116" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J117" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="J118" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="J119" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="J120" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J121" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="J122" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="J123" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="J124" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J125" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="J126" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="J127" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="J128" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="J129" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="J130" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="J131" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="J132" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="J133" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="J134" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="J135" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="J136" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="J137" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="J138" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="J139" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J140" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="J141" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="J142" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="J143" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="J144" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="J145" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1744,42 +2718,42 @@
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="91.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="91.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
-        <v>88</v>
+      <c r="A1" s="5" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
-        <v>89</v>
+      <c r="A2" s="5" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>90</v>
+      <c r="A3" s="4" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>91</v>
+      <c r="A4" s="4" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>92</v>
+      <c r="A6" s="5" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>93</v>
+      <c r="A8" s="4" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>94</v>
+      <c r="A9" s="3" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(sg): remove (SG) suffix for municipalities
Related to https://jira.sg.ch/browse/EBAU-203
</commit_message>
<xml_diff>
--- a/django/kt_sg/import/Services_SG.xlsx
+++ b/django/kt_sg/import/Services_SG.xlsx
@@ -68,7 +68,7 @@
     <t xml:space="preserve">Wittenbach</t>
   </si>
   <si>
-    <t xml:space="preserve">Berg (SG)</t>
+    <t xml:space="preserve">Berg</t>
   </si>
   <si>
     <t xml:space="preserve">Eggersriet</t>
@@ -95,7 +95,7 @@
     <t xml:space="preserve">Untereggen</t>
   </si>
   <si>
-    <t xml:space="preserve">Au (SG)</t>
+    <t xml:space="preserve">Au</t>
   </si>
   <si>
     <t xml:space="preserve">Balgach</t>
@@ -125,19 +125,19 @@
     <t xml:space="preserve">Eichberg</t>
   </si>
   <si>
-    <t xml:space="preserve">Marbach (SG)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oberriet (SG)</t>
+    <t xml:space="preserve">Marbach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oberriet</t>
   </si>
   <si>
     <t xml:space="preserve">Rebstein</t>
   </si>
   <si>
-    <t xml:space="preserve">Rüthi (SG)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buchs (SG)</t>
+    <t xml:space="preserve">Rüthi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buchs</t>
   </si>
   <si>
     <t xml:space="preserve">Gams</t>
@@ -182,7 +182,7 @@
     <t xml:space="preserve">Amden</t>
   </si>
   <si>
-    <t xml:space="preserve">Benken (SG)</t>
+    <t xml:space="preserve">Benken</t>
   </si>
   <si>
     <t xml:space="preserve">Kaltbrunn</t>
@@ -206,7 +206,7 @@
     <t xml:space="preserve">Gommiswald</t>
   </si>
   <si>
-    <t xml:space="preserve">Eschenbach (SG)</t>
+    <t xml:space="preserve">Eschenbach</t>
   </si>
   <si>
     <t xml:space="preserve">Ebnat-Kappel</t>
@@ -224,7 +224,7 @@
     <t xml:space="preserve">Wattwil</t>
   </si>
   <si>
-    <t xml:space="preserve">Kirchberg (SG)</t>
+    <t xml:space="preserve">Kirchberg</t>
   </si>
   <si>
     <t xml:space="preserve">Lütisburg</t>
@@ -263,19 +263,19 @@
     <t xml:space="preserve">Oberbüren</t>
   </si>
   <si>
-    <t xml:space="preserve">Zuzwil (SG)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wil (SG)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Andwil (SG)</t>
+    <t xml:space="preserve">Zuzwil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andwil</t>
   </si>
   <si>
     <t xml:space="preserve">Gaiserwald</t>
   </si>
   <si>
-    <t xml:space="preserve">Gossau (SG)</t>
+    <t xml:space="preserve">Gossau</t>
   </si>
   <si>
     <t xml:space="preserve">Waldkirch</t>

</xml_diff>